<commit_message>
Mistři early/play-off sezón dle PDF+web: doplnit/opravit M badge
- 1953/54: doplněn chybějící M → TJ Spartak Praha Sokolovo (vítěz finále)
- 1955/56: doplněn M → Rudá hvězda Brno (finále)
- 1975/76: doplněn M → SONP Kladno (finále)
- 1972/73: opraveno M Dukla Jihlava → Tesla Pardubice (první play-off, Tesla ve
  finále porazila Duklu 4:2 = první titul Pardubic; ověřeno webem). META měla pravdu.
</commit_message>
<xml_diff>
--- a/data/S1972_73_FINAL.xlsx
+++ b/data/S1972_73_FINAL.xlsx
@@ -719,6 +719,11 @@
           <t>Tesla Pardubice</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>36</v>
       </c>
@@ -795,11 +800,6 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>Dukla Jihlava</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>M</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -20420,7 +20420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20707,6 +20707,13 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>TODO-auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1972/73 první play-off: Tesla Pardubice (1. ZČ) ve finále porazila Duklu Jihlava 4:2 — první titul Pardubic. M badge opraven (byl chybně u Dukly). Doloženo webem.</t>
         </is>
       </c>
     </row>
@@ -21132,8 +21139,6 @@
           <t>NODE_S1972_73_0001</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21189,8 +21194,6 @@
           <t>NODE_S1972_73_0001</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21330,8 +21333,6 @@
           <t>NODE_S1972_73_0003</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -22255,8 +22256,6 @@
           <t>NODE_S1972_73_0026</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -22307,8 +22306,6 @@
           <t>NODE_S1972_73_0026</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23140,8 +23137,6 @@
           <t>NODE_S1972_73_0048</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23516,8 +23511,6 @@
           <t>NODE_S1972_73_0055</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24471,8 +24464,6 @@
           <t>NODE_S1972_73_0075</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25107,7 +25098,6 @@
           <t>NODE_S1972_73_0093</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25158,8 +25148,6 @@
           <t>NODE_S1972_73_0086</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -58963,7 +58951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59203,6 +59191,18 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Pro sezonu 1973/1974 vznikla 1. ČNHL (12 týmů) a 2. ČNHL (24 týmů ve 3 skupinách); přechodová logika převzata z PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mistr</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tesla Pardubice</t>
         </is>
       </c>
     </row>

</xml_diff>